<commit_message>
Switch to all_groups_final_annotated.csv — sub_topic now real
- build_data.py + upload_panel.jsx: point at all_groups_final_annotated.csv
- compute.py: normalize sub_topic (difflib-clusters LLM typo variants like
  'rủi ko/zo/ico' into canonical 'rủi ro' before downstream use)
- Q5/Q6 negative-topic breakdown now uses sub_topic when populated,
  falling back to master_topic when not (via _column_populated guard)
- Q3_SUBS auto-upgraded via existing _column_populated check — 24 real
  sub-topics instead of keyword-matched 19
- question_coverage.xlsx: Q3 / Q5 / Q6 flipped Pending → OK

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/question_coverage.xlsx
+++ b/question_coverage.xlsx
@@ -54,12 +54,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00E0E7FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0E7FF"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -553,29 +553,29 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Master + sub-topics: Seller vs Prospect</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>sub_topic × persona</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Keyword fallback today; real when sub_topic filled</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Real now (sub_topic 72% filled)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -607,108 +607,108 @@
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Q5</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Negative sub-topic × day of week</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>sub_topic × sentiment=negative × day</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Master-topic fallback today; real when sub_topic filled</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Real now (sub_topic 72% filled)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Q6</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Negative sub-topic × hour of day</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>sub_topic × sentiment=negative × hour</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Master-topic fallback today; real when sub_topic filled</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Real now (sub_topic 72% filled)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Q7</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Join triggers + benefits</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>content keywords + sentiment</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Keyword-based (permanent — no dedicated column)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Approx</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Abandonment signals + indicators</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>trigger_to_leave</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Keyword fallback today; real when trigger_to_leave filled</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -722,7 +722,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Active participants (persona) + KOLs</t>
+          <t>Active participants (persona donuts)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Real now (persona only, KOL individuals skipped)</t>
+          <t>Real now (persona donuts; KOL individuals skipped)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -742,162 +742,162 @@
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Q10</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Top product categories</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Product Category</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Keyword fallback today; real when Product Category filled</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Q11a</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Tool / program usage</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>brand_mentions</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Keyword fallback today; real when brand_mentions filled</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Q11b</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Satisfaction vs issues per tool</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>sentiment × brand_mentions (cross-tab)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Approximation — post-level sentiment as proxy for per-tool sentiment</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Approx</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Q12</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>3rd-party outsourcing services</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>content keywords (or brand_mentions if LLM puts service names there)</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Keyword-based (permanent — no dedicated column)</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Approx</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Q13</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Amazon courses sellers want</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>content keywords (or brand_mentions if LLM puts course names there)</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Keyword-based (permanent — no dedicated column)</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Approx</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Q14</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Business growth + P&amp;L polarity</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>content keywords + sentiment + P&amp;L regex cross-tab</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Approximation — post-level sentiment as proxy for P&amp;L polarity</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Approx</t>
         </is>

</xml_diff>